<commit_message>
diferenciador a pulsera inteligente
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
+++ b/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
@@ -605,7 +605,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1102,7 +1101,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Botón de asistencia (App). Modo "pantalla en casa" sobre tablet fija (App)</t>
+          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Integración de pulsera inteligente: ubicación, salud y funciones de seguridad (BD + Backend + App)</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1138,7 +1137,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Módulo de IA — orientación general (integración API LLM) y detección simple de patrones (BD + IA). Integración con pulsera inteligente vía Health Connect (BD + Backend)</t>
+          <t>Módulo de IA — orientación general (integración API LLM). Registro manual de glucosa y recordatorios extendidos (post-consulta médica y citas pendientes)</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -1174,7 +1173,7 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Detección de sonidos fuertes vía micrófono del dispositivo (App). Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
+          <t>Farmacias cercanas vía IA (comparación de precio y cercanía). Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
@@ -1312,7 +1311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1729,7 +1728,7 @@
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Como perfil dependiente (ej. adulto mayor) quiero una interfaz simplificada con botones grandes y confirmación en un toque, disponible también en modo "pantalla en casa" sobre una tablet fija (vía Fully Kiosk Browser) para quienes no manejan un smartphone</t>
+          <t>Como perfil dependiente (ej. adulto mayor) quiero una interfaz simplificada con botones grandes y confirmación en un toque</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -1934,17 +1933,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pulsera inteligente</t>
+          <t>Pulsera: ubicación</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Como titular o cuidador quiero ver signos vitales (frecuencia cardíaca) de un perfil desde una pulsera inteligente conectada, sin instrumentación adicional</t>
+          <t>Como titular o cuidador quiero ver la ubicación en tiempo real y recibir alertas de geocerca (colegio, casa) desde la pulsera del perfil dependiente</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Perfil (titular/dependiente)</t>
+          <t>Perfil dependiente (niño/adulto mayor)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1959,7 +1958,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
@@ -1969,12 +1968,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Detección de ruido</t>
+          <t>Pulsera: salud</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Como cuidador quiero recibir una alerta si el dispositivo del perfil dependiente detecta un sonido fuerte en el hogar (posible caída)</t>
+          <t>Como titular o cuidador quiero ver frecuencia cardíaca y presión referencial del perfil dependiente desde la pulsera conectada</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1984,17 +1983,157 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Matías (App) / Benjamín (Backend)</t>
+          <t>Sergio (BD) / Benjamín (Backend)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Pulsera: seguridad</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Como cuidador quiero recibir una alerta si la pulsera detecta una caída, se presiona el botón SOS, la batería está baja, o hay inactividad inusual</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Perfil dependiente</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Benjamín (Backend) / Matías (App)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Registro manual de glucosa</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Como cuidador quiero ingresar manualmente la lectura de un glucómetro certificado y verla en el historial del perfil</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Perfil dependiente diabético</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Matías (App) / Sergio (BD)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Sprint 6</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Recordatorios extendidos</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Como cuidador quiero registrar indicaciones post-consulta médica y citas médicas pendientes, con recordatorio diario hasta la fecha</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Titular / Cuidador</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Benjamín (Backend)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Farmacias cercanas vía IA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Como usuario quiero preguntarle a la IA por un medicamento y que me recomiende farmacias cercanas comparando precio</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Titular / Cuidador</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sergio (BD) / Benjamín (Backend)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Baja</t>
         </is>
       </c>
     </row>
@@ -2029,6 +2168,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2113,10 +2253,11 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Diseño e implementación de la interfaz para paciente, adulto mayor y cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
-        </is>
-      </c>
-    </row>
+          <t>Diseño e implementación de la interfaz para el titular, el perfil dependiente y el cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Integra Traccar para GPS propio
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
+++ b/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
@@ -605,6 +605,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1101,7 +1102,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Integración de pulsera inteligente: ubicación, salud y funciones de seguridad (BD + Backend + App)</t>
+          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Integración de pulsera: servidor Traccar (GPS/geocercas) + Health Connect (salud) + funciones de seguridad (BD + Backend + App)</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1330,6 +1331,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1938,7 +1940,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Como titular o cuidador quiero ver la ubicación en tiempo real y recibir alertas de geocerca (colegio, casa) desde la pulsera del perfil dependiente</t>
+          <t>Como titular o cuidador quiero ver la ubicación en tiempo real y recibir alertas de geocerca (colegio, casa) desde la pulsera, vía un servidor Traccar propio (open source) que recibe el GPS directo del dispositivo, sin depender de la app del fabricante</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2168,7 +2170,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2253,11 +2254,10 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Diseño e implementación de la interfaz para el titular, el perfil dependiente y el cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
+          <t>Diseño e implementación de la interfaz para el titular, el perfil dependiente (persona no valente) y el cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Cronograma: nombres de documentos oficiales, formativas, retrospectivas y plan por sprint al día
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
+++ b/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
@@ -605,7 +605,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -711,7 +710,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>1.3 Autoevaluación Fase 1 + Cronograma de actividades del equipo</t>
+          <t>1.3 Autoevaluación Fase 1 + 1.4 Formativa Fase 1 (grupal, sin nota) + Cronograma de actividades del equipo</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -855,7 +854,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>Módulo de autenticación funcional</t>
+          <t>Módulo de autenticación funcional + Demo interna Sprint 1 + Retrospectiva</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -891,7 +890,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>Sprint Backlog 2 + avance módulo rutinas</t>
+          <t>Sprint Backlog 2 + avance módulo rutinas + 2.3 Formativa Informe de avance (grupal, sin nota)</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -922,7 +921,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Confirmación de actividades end-to-end: API, BD y UI conectadas</t>
+          <t>Confirmación de actividades: agenda diaria en la app y API. El guardado de la confirmación en el servidor (tabla ACTIVIDAD) se completa en el Sprint 3</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -958,12 +957,12 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Creación y vinculación de perfiles dependientes a la cuenta titular, e invitación de cuidadores adicionales con permisos configurables (Backend + BD). Panel de gestión de dependientes (App) — versión inicial</t>
+          <t>Creación y vinculación de perfiles dependientes a la cuenta titular, e invitación de cuidadores adicionales con permisos configurables (Backend + BD). Cierre de la confirmación de actividades guardada en el servidor (tabla ACTIVIDAD). Panel de gestión de dependientes (App) — versión inicial</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Sprint Backlog 3 + Autoevaluación avance Fase 2</t>
+          <t>Sprint Backlog 3 + 2.1 Diario de Reflexión Fase 2 + 2.2 Autoevaluación avance Fase 2</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -994,12 +993,12 @@
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Cierre de Sprint 3 e integración. Preparación y entrega del Informe de Avance del Proyecto APT</t>
+          <t>Cierre de Sprint 3 e integración (pruebas de la app y del backend, aceptación del Product Owner). Preparación y entrega del Informe de Avance del Proyecto APT</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>2.5 Sumativa Avance Fase 2 (20%) — Informe de avance</t>
+          <t>2.4 Sumativa Avance Fase 2 (20%) — Informe de avance + Retrospectiva Sprint 3</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1030,12 +1029,12 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Retroalimentación del avance. Sistema de recordatorios y notificaciones push (Backend + App)</t>
+          <t>Retroalimentación del avance. RUTINA_HORARIO y generación programada de actividades. Sistema de recordatorios y notificaciones push (Backend + App)</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>Sprint Backlog 4 + Retrospectiva</t>
+          <t>Sprint Backlog 4</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -1066,12 +1065,12 @@
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Sistema de alertas hacia titular/cuidadores + interfaz simplificada para perfiles dependientes (App). Indicadores de salud (BD)</t>
+          <t>Sistema de alertas escalonadas hacia titular/cuidadores + interfaz simplificada para perfiles dependientes (App)</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Demo interna Sprint 4</t>
+          <t>Demo interna Sprint 4 + Retrospectiva</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1102,7 +1101,7 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Historial de cumplimiento y gráficos de indicadores (BD + Backend). Integración de pulsera: servidor Traccar (GPS/geocercas) + Health Connect (salud) + funciones de seguridad (BD + Backend + App)</t>
+          <t>Indicadores de salud (peso, presión, glucosa), historial de cumplimiento y gráficos (BD + Backend). Integración de pulsera: servidor Traccar (GPS/geocercas) + Health Connect (salud) + funciones de seguridad y botón "Necesito ayuda" (BD + Backend + App)</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
@@ -1138,7 +1137,7 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Módulo de IA — orientación general (integración API LLM). Registro manual de glucosa y recordatorios extendidos (post-consulta médica y citas pendientes)</t>
+          <t>Módulo de IA — orientación general (integración API LLM). Cierre e integración de la pulsera</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
@@ -1174,12 +1173,12 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Farmacias cercanas vía IA (comparación de precio y cercanía). Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
+          <t>Registro manual de glucosa y recordatorios extendidos (post-consulta médica y citas pendientes). Farmacias cercanas vía IA (comparación de precio y cercanía). Pruebas integrales, ajustes finales, documentación (manual técnico, Docker) y presentación del Informe Final</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>2.7 Sumativa Final Fase 2 (30%) — Informe final + demo</t>
+          <t>2.6 Sumativa Final Fase 2 (30%) — Informe final + demo + Retrospectiva Sprint 6</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
@@ -1312,7 +1311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1322,6 +1321,7 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1331,7 +1331,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1366,6 +1365,11 @@
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Prioridad</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Estado real (al 17-10-2026)</t>
         </is>
       </c>
     </row>
@@ -1403,6 +1407,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>Terminada en el Sprint 1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="n">
@@ -1438,6 +1447,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>Terminada en el Sprint 2 (parte parcial desde el Sprint 1)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="19" t="n">
@@ -1473,6 +1487,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>Terminada en el Sprint 2 (app el 10-10)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="n">
@@ -1508,6 +1527,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Terminada en el Sprint 2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="n">
@@ -1530,7 +1554,7 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Matías (App)</t>
+          <t>Matías (App) / Benjamín (Backend) / Sergio (BD)</t>
         </is>
       </c>
       <c r="F8" s="19" t="inlineStr">
@@ -1541,6 +1565,11 @@
       <c r="G8" s="19" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>Terminada en el Sprint 2; confirmación en el servidor en el Sprint 3</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1594,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>Benjamín (Backend) / Sergio (BD)</t>
+          <t>Benjamín (Backend) / Matías (App) / Sergio (BD)</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -1576,6 +1605,11 @@
       <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 3: lista, falta la aceptación del PO</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1634,7 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Benjamín (Backend) / Sergio (BD)</t>
+          <t>Benjamín (Backend) / Matías (App) / Sergio (BD)</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
@@ -1611,6 +1645,11 @@
       <c r="G10" s="19" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 3: lista, falta la aceptación del PO</t>
         </is>
       </c>
     </row>
@@ -1648,6 +1687,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 3: lista, falta la aceptación del PO</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="n">
@@ -1683,6 +1727,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="n">
@@ -1718,6 +1767,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="n">
@@ -1753,6 +1807,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="n">
@@ -1788,6 +1847,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="n">
@@ -1823,6 +1887,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="n">
@@ -1858,6 +1927,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n">
@@ -1893,6 +1967,11 @@
           <t>Baja</t>
         </is>
       </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="n">
@@ -1928,6 +2007,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1963,6 +2047,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1998,6 +2087,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2033,6 +2127,11 @@
           <t>Alta</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2068,6 +2167,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2103,6 +2207,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2136,6 +2245,11 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>Baja</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
@@ -2254,14 +2368,14 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Diseño e implementación de la interfaz para el titular, el perfil dependiente (persona no valente) y el cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Diseño e implementación de la interfaz para el titular, el perfil dependiente (persona no autovalente) y el cuidador, experiencia de usuario accesible, manejo de notificaciones en el cliente y consumo de la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Nota: aunque cada integrante es dueño principal de un módulo, todas las tareas de integración, pruebas, documentación (README, manual técnico) y la presentación final son responsabilidad compartida del equipo.</t>
+          <t>Nota: aunque cada integrante es dueño principal de un módulo, todas las tareas de integración, pruebas, documentación (README, manual técnico) y la presentación final son responsabilidad compartida del equipo. Roles Scrum: Matías Pizarro es Scrum Master y Sergio Ocares es Product Owner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cronograma: demo interna al cierre de cada sprint y demo final en Fase 3, según la Guía Sumativa Fase 1
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
+++ b/Fase 1/Evidencias Grupales/Cronograma_Actividades_Equipo_PerfilMedico.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>2.4 Sumativa Avance Fase 2 (20%) — Informe de avance + Retrospectiva Sprint 3</t>
+          <t>2.4 Sumativa Avance Fase 2 (20%) — Informe de avance + Demo interna y Retrospectiva Sprint 3</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>2.6 Sumativa Final Fase 2 (30%) — Informe final + demo + Retrospectiva Sprint 6</t>
+          <t>2.6 Sumativa Final Fase 2 (30%) — Informe final + manual técnico + README + aplicación funcional con backend en Docker. Demo interna y Retrospectiva Sprint 6</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>Ensayo grupal + material de apoyo</t>
+          <t>Ensayo grupal + material de apoyo + demo</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>Presentación y defensa final del Proyecto APT ante comisión calificadora</t>
+          <t>Presentación y demo final del Proyecto APT, y defensa ante comisión calificadora</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">

</xml_diff>